<commit_message>
Update SportMatch Excel file with latest data revisions
</commit_message>
<xml_diff>
--- a/outputs/SportMatch - Equipo 11 - EVM y Curva S.xlsx
+++ b/outputs/SportMatch - Equipo 11 - EVM y Curva S.xlsx
@@ -502,7 +502,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
@@ -624,9 +624,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="10" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -1679,12 +1676,73 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Curva S'!$B$5:$B$17</c:f>
+              <c:f>'Curva S'!$B$5:$B$16</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>13/08</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20/08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27/08</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>03/09</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10/09</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>17/09</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>24/09</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>01/10</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>08/10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>15/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>22/10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>29/10</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>PRESUPUESTO!$B$44:$G$44</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>420</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>793.14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1033.14</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1213.14</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
@@ -1758,12 +1816,73 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Curva S'!$B$5:$B$17</c:f>
+              <c:f>'Curva S'!$B$5:$B$16</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>13/08</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20/08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27/08</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>03/09</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10/09</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>17/09</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>24/09</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>01/10</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>08/10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>15/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>22/10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>29/10</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>PRESUPUESTO!$B$42:$G$42</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>440</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>640</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>863.14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1133.14</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1363.14</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
@@ -1788,12 +1907,91 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'Curva S'!$B$5:$B$17</c:f>
+              <c:f>'Curva S'!$B$5:$B$16</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>13/08</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20/08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27/08</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>03/09</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10/09</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>17/09</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>24/09</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>01/10</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>08/10</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>15/10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>22/10</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>29/10</c:v>
+                </c:pt>
+              </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>PRESUPUESTO!$B$40:$N$40</c:f>
+              <c:f>PRESUPUESTO!$B$40:$M$40</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>420</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>793.14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1033.14</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1213.14</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1393.14</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1586.28</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1766.28</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2006.28</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2186.28</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2379.42</c:v>
+                </c:pt>
+              </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
@@ -3881,9 +4079,7 @@
       <c r="M9" s="50">
         <v>60</v>
       </c>
-      <c r="N9" s="50">
-        <v>60</v>
-      </c>
+      <c r="N9" s="50"/>
       <c r="O9" s="50"/>
       <c r="P9" s="50"/>
       <c r="Q9" s="50"/>
@@ -3897,6 +4093,7 @@
       <c r="Y9" s="50"/>
       <c r="Z9" s="51">
         <f t="shared" ref="Z9:Z33" si="0">SUM(B9:Y9)</f>
+        <v>720</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
@@ -3941,9 +4138,7 @@
       <c r="M10" s="50">
         <v>60</v>
       </c>
-      <c r="N10" s="50">
-        <v>60</v>
-      </c>
+      <c r="N10" s="50"/>
       <c r="O10" s="50"/>
       <c r="P10" s="50"/>
       <c r="Q10" s="50"/>
@@ -4002,9 +4197,7 @@
       <c r="M11" s="50">
         <v>60</v>
       </c>
-      <c r="N11" s="50">
-        <v>60</v>
-      </c>
+      <c r="N11" s="50"/>
       <c r="O11" s="50"/>
       <c r="P11" s="50"/>
       <c r="Q11" s="50"/>
@@ -4714,6 +4907,7 @@
       </c>
       <c r="B34" s="52">
         <f t="shared" ref="B34:Z34" si="1">SUM(B9:B33)</f>
+        <v>240</v>
       </c>
       <c r="C34" s="52">
         <f t="shared" si="1"/>
@@ -4826,6 +5020,7 @@
       </c>
       <c r="D35" s="52">
         <f t="shared" ref="D35:G35" si="2">C35+D34</f>
+        <v>600</v>
       </c>
       <c r="E35" s="52">
         <f t="shared" si="2"/>
@@ -4841,37 +5036,47 @@
       </c>
       <c r="H35" s="52">
         <f t="shared" ref="H35" si="3">G35+H34</f>
+        <v>1393.14</v>
       </c>
       <c r="I35" s="52">
         <f t="shared" ref="I35" si="4">H35+I34</f>
+        <v>1586.28</v>
       </c>
       <c r="J35" s="52">
         <f t="shared" ref="J35" si="5">I35+J34</f>
+        <v>1766.28</v>
       </c>
       <c r="K35" s="52">
         <f t="shared" ref="K35" si="6">J35+K34</f>
+        <v>2006.28</v>
       </c>
       <c r="L35" s="52">
         <f t="shared" ref="L35" si="7">K35+L34</f>
+        <v>2186.28</v>
       </c>
       <c r="M35" s="52">
         <f t="shared" ref="M35" si="8">L35+M34</f>
+        <v>2379.42</v>
       </c>
       <c r="N35" s="52">
         <f t="shared" ref="N35" si="9">M35+N34</f>
+        <v>2379.42</v>
       </c>
       <c r="O35" s="52">
         <f t="shared" ref="O35" si="10">N35+O34</f>
+        <v>2379.42</v>
       </c>
       <c r="P35" s="52">
         <f t="shared" ref="P35" si="11">O35+P34</f>
+        <v>2379.42</v>
       </c>
       <c r="Q35" s="52">
         <f>P35+Q34</f>
-        <v>2559.4199999999996</v>
+        <v>2379.42</v>
       </c>
       <c r="R35" s="52">
         <f t="shared" ref="R35:W35" si="12">Q35+R34</f>
+        <v>2379.42</v>
       </c>
       <c r="S35" s="52">
         <f t="shared" si="12"/>
@@ -4895,11 +5100,11 @@
       </c>
       <c r="X35" s="52">
         <f>W35+X34</f>
-        <v>2559.4199999999996</v>
+        <v>2379.42</v>
       </c>
       <c r="Y35" s="52">
         <f>X35+Y34</f>
-        <v>2559.4199999999996</v>
+        <v>2379.42</v>
       </c>
     </row>
     <row r="38" spans="1:26" ht="16.5" x14ac:dyDescent="0.25">
@@ -4912,6 +5117,7 @@
       </c>
       <c r="C38" s="16">
         <f t="shared" ref="C38:G38" si="13">C34</f>
+        <v>180</v>
       </c>
       <c r="D38" s="16">
         <f t="shared" si="13"/>
@@ -4931,6 +5137,7 @@
       </c>
       <c r="H38" s="16">
         <f t="shared" ref="H38:Y38" si="14">H34</f>
+        <v>180</v>
       </c>
       <c r="I38" s="16">
         <f t="shared" si="14"/>
@@ -4942,6 +5149,7 @@
       </c>
       <c r="K38" s="16">
         <f t="shared" ref="K38:X38" si="15">K34</f>
+        <v>240</v>
       </c>
       <c r="L38" s="16">
         <f t="shared" si="15"/>
@@ -4969,6 +5177,7 @@
       </c>
       <c r="R38" s="16">
         <f t="shared" ref="R38:W38" si="16">R34</f>
+        <v>0</v>
       </c>
       <c r="S38" s="16">
         <f t="shared" si="16"/>
@@ -5012,6 +5221,7 @@
       </c>
       <c r="C39" s="22">
         <f t="shared" ref="C39:Y39" si="17">C38</f>
+        <v>180</v>
       </c>
       <c r="D39" s="22">
         <f t="shared" si="17"/>
@@ -5103,7 +5313,7 @@
       </c>
       <c r="Z39" s="20">
         <f>Z34</f>
-        <v>2559.42</v>
+        <v>2379.42</v>
       </c>
     </row>
     <row r="40" spans="1:26" x14ac:dyDescent="0.25">
@@ -5116,6 +5326,7 @@
       </c>
       <c r="C40" s="11">
         <f t="shared" ref="C40:G40" si="18">C35</f>
+        <v>420</v>
       </c>
       <c r="D40" s="11">
         <f>D35</f>
@@ -5135,6 +5346,7 @@
       </c>
       <c r="H40" s="11">
         <f t="shared" ref="H40:Y40" si="19">H35</f>
+        <v>1393.14</v>
       </c>
       <c r="I40" s="11">
         <f t="shared" si="19"/>
@@ -5146,6 +5358,7 @@
       </c>
       <c r="K40" s="11">
         <f t="shared" ref="K40:X40" si="20">K35</f>
+        <v>2006.28</v>
       </c>
       <c r="L40" s="11">
         <f t="shared" si="20"/>
@@ -5173,6 +5386,7 @@
       </c>
       <c r="R40" s="11">
         <f t="shared" ref="R40:W40" si="21">R35</f>
+        <v>2379.42</v>
       </c>
       <c r="S40" s="11">
         <f t="shared" si="21"/>
@@ -5209,27 +5423,27 @@
       </c>
       <c r="B41" s="21">
         <f>'Avance semanal'!J6</f>
-        <v>63.51777817886472</v>
+        <v>140</v>
       </c>
       <c r="C41" s="21">
         <f>'Avance semanal'!J7</f>
-        <v>377.75754986012095</v>
+        <v>300</v>
       </c>
       <c r="D41" s="21">
         <f>'Avance semanal'!J8</f>
-        <v>100.70455013085463</v>
+        <v>200</v>
       </c>
       <c r="E41" s="21">
         <f>'Avance semanal'!J9</f>
-        <v>349.9252143308365</v>
+        <v>223.14</v>
       </c>
       <c r="F41" s="21">
         <f>'Avance semanal'!J10</f>
-        <v>303.6149796949734</v>
+        <v>270</v>
       </c>
       <c r="G41" s="21">
         <f>'Avance semanal'!J11</f>
-        <v>214.22814276689832</v>
+        <v>230</v>
       </c>
       <c r="H41" s="21"/>
       <c r="I41" s="21"/>
@@ -5256,14 +5470,15 @@
       </c>
       <c r="B42" s="12">
         <f>IF(B41=0,NA(),B41)</f>
-        <v>63.51777817886472</v>
+        <v>140</v>
       </c>
       <c r="C42" s="12">
         <f>IF(C41=0,NA(),B42+C41)</f>
-        <v>441.27532803898566</v>
+        <v>440</v>
       </c>
       <c r="D42" s="12">
         <f t="shared" ref="D42:Y42" si="22">IF(D41=0,NA(),C42+D41)</f>
+        <v>640</v>
       </c>
       <c r="E42" s="12">
         <f t="shared" si="22"/>
@@ -5411,6 +5626,7 @@
       </c>
       <c r="D44" s="13">
         <f t="shared" ref="D44:Y44" si="23">IF(D41=0,NA(),C44+D43)</f>
+        <v>600</v>
       </c>
       <c r="E44" s="13">
         <f t="shared" si="23"/>
@@ -5503,6 +5719,7 @@
       </c>
       <c r="B45" s="14">
         <f t="shared" ref="B45:Y45" si="24">IFERROR(B42/B40,"-")</f>
+        <v>0.5833333333</v>
       </c>
       <c r="C45" s="14">
         <f t="shared" si="24"/>
@@ -5603,10 +5820,11 @@
       </c>
       <c r="B46" s="14">
         <f>IFERROR(B42/B44,"-")</f>
-        <v>0.26465740907860297</v>
+        <v>0.5833333333</v>
       </c>
       <c r="C46" s="14">
         <f t="shared" ref="C46:Y46" si="25">IFERROR(C42/C44,"-")</f>
+        <v>1.0476190476</v>
       </c>
       <c r="D46" s="14">
         <f t="shared" si="25"/>
@@ -5638,6 +5856,7 @@
       </c>
       <c r="K46" s="14" t="str">
         <f t="shared" ref="K46:X46" si="26">IFERROR(K42/K44,"-")</f>
+        <v>-</v>
       </c>
       <c r="L46" s="14" t="str">
         <f t="shared" si="26"/>
@@ -5665,6 +5884,7 @@
       </c>
       <c r="R46" s="14" t="str">
         <f t="shared" ref="R46:W46" si="27">IFERROR(R42/R44,"-")</f>
+        <v>-</v>
       </c>
       <c r="S46" s="14" t="str">
         <f t="shared" si="27"/>
@@ -5942,7 +6162,7 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equipo 11 · Corte 17/09/2026 (semana 6, cierre del S1) · USD acumulados (devs + infra + IA) · Base: WBS y Cronograma v4 · Datos desde PRESUPUESTO y Avance semanal</t>
+          <t xml:space="preserve">Equipo 11 · Corte 17/09/2026 (semana 6) · USD acumulados (devs + infra + IA) · Datos desde PRESUPUESTO y Avance semanal</t>
         </is>
       </c>
     </row>
@@ -6010,7 +6230,7 @@
       </c>
       <c r="C5" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1 · Capacitación</t>
+          <t xml:space="preserve">Capacitación</t>
         </is>
       </c>
       <c r="D5" s="28">
@@ -6019,7 +6239,7 @@
       </c>
       <c r="E5" s="28">
         <f>IFERROR(PRESUPUESTO!B42,"")</f>
-        <v>63.51777817886472</v>
+        <v>140</v>
       </c>
       <c r="F5" s="28">
         <f>IFERROR(PRESUPUESTO!B44,"")</f>
@@ -6031,7 +6251,7 @@
       </c>
       <c r="H5" s="29">
         <f>SUM('Avance semanal'!$F$6:F6)</f>
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="I5" s="29">
         <f>SUM('Avance semanal'!$E$6:E6)</f>
@@ -6057,7 +6277,7 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 1</t>
         </is>
       </c>
       <c r="D6" s="28">
@@ -6066,7 +6286,7 @@
       </c>
       <c r="E6" s="28">
         <f>IFERROR(PRESUPUESTO!C42,"")</f>
-        <v>441.27532803898566</v>
+        <v>440</v>
       </c>
       <c r="F6" s="28">
         <f>IFERROR(PRESUPUESTO!C44,"")</f>
@@ -6078,7 +6298,7 @@
       </c>
       <c r="H6" s="29">
         <f>SUM('Avance semanal'!$F$6:F7)</f>
-        <v>38.21</v>
+        <v>38</v>
       </c>
       <c r="I6" s="29">
         <f>SUM('Avance semanal'!$E$6:E7)</f>
@@ -6104,7 +6324,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 2</t>
         </is>
       </c>
       <c r="D7" s="28">
@@ -6113,7 +6333,7 @@
       </c>
       <c r="E7" s="28">
         <f>IFERROR(PRESUPUESTO!D42,"")</f>
-        <v>541.9798781698403</v>
+        <v>640</v>
       </c>
       <c r="F7" s="28">
         <f>IFERROR(PRESUPUESTO!D44,"")</f>
@@ -6125,7 +6345,7 @@
       </c>
       <c r="H7" s="29">
         <f>SUM('Avance semanal'!$F$6:F8)</f>
-        <v>46.93</v>
+        <v>58</v>
       </c>
       <c r="I7" s="29">
         <f>SUM('Avance semanal'!$E$6:E8)</f>
@@ -6137,7 +6357,7 @@
         </is>
       </c>
       <c r="L7" s="31">
-        <v>8063.3</v>
+        <v>11221.2</v>
       </c>
     </row>
     <row r="8">
@@ -6151,7 +6371,7 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 3</t>
         </is>
       </c>
       <c r="D8" s="28">
@@ -6160,7 +6380,7 @@
       </c>
       <c r="E8" s="28">
         <f>IFERROR(PRESUPUESTO!E42,"")</f>
-        <v>891.9050925006768</v>
+        <v>863.14</v>
       </c>
       <c r="F8" s="28">
         <f>IFERROR(PRESUPUESTO!E44,"")</f>
@@ -6172,7 +6392,7 @@
       </c>
       <c r="H8" s="29">
         <f>SUM('Avance semanal'!$F$6:F9)</f>
-        <v>77.23</v>
+        <v>79</v>
       </c>
       <c r="I8" s="29">
         <f>SUM('Avance semanal'!$E$6:E9)</f>
@@ -6185,7 +6405,7 @@
       </c>
       <c r="L8" s="38">
         <f>PRESUPUESTO!Z39</f>
-        <v>2559.42</v>
+        <v>2379.42</v>
       </c>
     </row>
     <row r="9">
@@ -6199,20 +6419,20 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 4</t>
         </is>
       </c>
       <c r="D9" s="28">
         <f>PRESUPUESTO!F40</f>
-        <v>1033.1399999999999</v>
+        <v>1033.14</v>
       </c>
       <c r="E9" s="28">
         <f>IFERROR(PRESUPUESTO!F42,"")</f>
-        <v>1195.5200721956503</v>
+        <v>1133.14</v>
       </c>
       <c r="F9" s="28">
         <f>IFERROR(PRESUPUESTO!F44,"")</f>
-        <v>1033.1399999999999</v>
+        <v>1033.14</v>
       </c>
       <c r="G9" s="29">
         <f>SUM('Avance semanal'!$D$6:D10)</f>
@@ -6220,20 +6440,12 @@
       </c>
       <c r="H9" s="29">
         <f>SUM('Avance semanal'!$F$6:F10)</f>
-        <v>103.52000000000001</v>
+        <v>100</v>
       </c>
       <c r="I9" s="29">
         <f>SUM('Avance semanal'!$E$6:E10)</f>
         <v>90</v>
       </c>
-      <c r="K9" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Esfuerzo de desarrollo (h, Cronograma v4)</t>
-        </is>
-      </c>
-      <c r="L9" s="30">
-        <v>221.62</v>
-      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="41">
@@ -6246,20 +6458,20 @@
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1 · CORTE (steering 1)</t>
+          <t xml:space="preserve">Sprint 5 · CORTE</t>
         </is>
       </c>
       <c r="D10" s="42">
         <f>PRESUPUESTO!G40</f>
-        <v>1213.1399999999999</v>
+        <v>1213.14</v>
       </c>
       <c r="E10" s="42">
         <f>IFERROR(PRESUPUESTO!G42,"")</f>
-        <v>1409.7482149625487</v>
+        <v>1363.14</v>
       </c>
       <c r="F10" s="42">
         <f>IFERROR(PRESUPUESTO!G44,"")</f>
-        <v>1213.1399999999999</v>
+        <v>1213.14</v>
       </c>
       <c r="G10" s="43">
         <f>SUM('Avance semanal'!$D$6:D11)</f>
@@ -6267,7 +6479,7 @@
       </c>
       <c r="H10" s="43">
         <f>SUM('Avance semanal'!$F$6:F11)</f>
-        <v>122.07000000000001</v>
+        <v>123</v>
       </c>
       <c r="I10" s="43">
         <f>SUM('Avance semanal'!$E$6:E11)</f>
@@ -6305,12 +6517,12 @@
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D11" s="28">
         <f>PRESUPUESTO!H40</f>
-        <v>1393.1399999999999</v>
+        <v>1393.14</v>
       </c>
       <c r="E11" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!H42,"")</f>
@@ -6333,10 +6545,10 @@
       </c>
       <c r="L11" s="38">
         <f>INDEX(PRESUPUESTO!$B$40:$Y$40,$L$5)</f>
-        <v>1213.1399999999999</v>
+        <v>1213.14</v>
       </c>
       <c r="M11" s="35">
-        <f>INDEX($G$5:$G$17,$L$5)</f>
+        <f>INDEX($G$5:$G$16,$L$5)</f>
         <v>108</v>
       </c>
       <c r="N11" s="39"/>
@@ -6352,12 +6564,12 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D12" s="28">
         <f>PRESUPUESTO!I40</f>
-        <v>1586.2799999999997</v>
+        <v>1586.28</v>
       </c>
       <c r="E12" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!I42,"")</f>
@@ -6380,11 +6592,11 @@
       </c>
       <c r="L12" s="38">
         <f>INDEX(PRESUPUESTO!$B$42:$Y$42,$L$5)</f>
-        <v>1409.7482149625487</v>
+        <v>1363.14</v>
       </c>
       <c r="M12" s="35">
-        <f>INDEX($H$5:$H$17,$L$5)</f>
-        <v>122.07000000000001</v>
+        <f>INDEX($H$5:$H$16,$L$5)</f>
+        <v>123</v>
       </c>
       <c r="N12" s="39"/>
     </row>
@@ -6399,12 +6611,12 @@
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D13" s="28">
         <f>PRESUPUESTO!J40</f>
-        <v>1766.2799999999997</v>
+        <v>1766.28</v>
       </c>
       <c r="E13" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!J42,"")</f>
@@ -6427,10 +6639,10 @@
       </c>
       <c r="L13" s="38">
         <f>INDEX(PRESUPUESTO!$B$44:$Y$44,$L$5)</f>
-        <v>1213.1399999999999</v>
+        <v>1213.14</v>
       </c>
       <c r="M13" s="35">
-        <f>INDEX($I$5:$I$17,$L$5)</f>
+        <f>INDEX($I$5:$I$16,$L$5)</f>
         <v>108</v>
       </c>
       <c r="N13" s="39"/>
@@ -6446,12 +6658,12 @@
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2 · MVP</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D14" s="28">
         <f>PRESUPUESTO!K40</f>
-        <v>2006.2799999999997</v>
+        <v>2006.28</v>
       </c>
       <c r="E14" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!K42,"")</f>
@@ -6474,11 +6686,11 @@
       </c>
       <c r="L14" s="33">
         <f>L12-L13</f>
-        <v>196.6082149625488</v>
+        <v>150</v>
       </c>
       <c r="M14" s="35">
         <f>M12-M13</f>
-        <v>14.070000000000007</v>
+        <v>15</v>
       </c>
       <c r="N14" s="39" t="str">
         <f>IF(L14&gt;=0,"Bajo presupuesto","Sobre presupuesto")</f>
@@ -6496,12 +6708,12 @@
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S3</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D15" s="28">
         <f>PRESUPUESTO!L40</f>
-        <v>2186.2799999999997</v>
+        <v>2186.28</v>
       </c>
       <c r="E15" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!L42,"")</f>
@@ -6524,11 +6736,11 @@
       </c>
       <c r="L15" s="33">
         <f>L12-L11</f>
-        <v>196.6082149625488</v>
+        <v>150</v>
       </c>
       <c r="M15" s="35">
         <f>M12-M11</f>
-        <v>14.070000000000007</v>
+        <v>15</v>
       </c>
       <c r="N15" s="39" t="str">
         <f>IF(L15&gt;=0,"Adelantado al plan","Atrasado")</f>
@@ -6546,12 +6758,12 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S3</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D16" s="28">
         <f>PRESUPUESTO!M40</f>
-        <v>2379.4199999999996</v>
+        <v>2379.42</v>
       </c>
       <c r="E16" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!M42,"")</f>
@@ -6574,7 +6786,7 @@
       </c>
       <c r="L16" s="34">
         <f>L12/L13</f>
-        <v>1.1620655612398807</v>
+        <v>1.1236460755</v>
       </c>
       <c r="M16" s="35"/>
       <c r="N16" s="39" t="str">
@@ -6583,35 +6795,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27">
-        <v>13</v>
-      </c>
-      <c r="B17" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">05/11</t>
-        </is>
-      </c>
-      <c r="C17" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S3 · Fin del desarrollo</t>
-        </is>
-      </c>
-      <c r="D17" s="28">
-        <f>PRESUPUESTO!N40</f>
-        <v>2559.4199999999996</v>
-      </c>
-      <c r="E17" s="28" t="str">
-        <f>IFERROR(PRESUPUESTO!N42,"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="28" t="str">
-        <f>IFERROR(PRESUPUESTO!N44,"")</f>
-        <v/>
-      </c>
-      <c r="G17" s="29">
-        <f>SUM('Avance semanal'!$D$6:D18)</f>
-        <v>234</v>
-      </c>
       <c r="K17" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">SPI = EV / PV</t>
@@ -6619,7 +6802,7 @@
       </c>
       <c r="L17" s="34">
         <f>L12/L11</f>
-        <v>1.1620655612398807</v>
+        <v>1.1236460755</v>
       </c>
       <c r="M17" s="35"/>
       <c r="N17" s="39" t="str">
@@ -6635,12 +6818,12 @@
       </c>
       <c r="K18" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">EAC = BAC EVM / CPI</t>
+          <t xml:space="preserve">EAC = BAC total / CPI</t>
         </is>
       </c>
       <c r="L18" s="33">
-        <f>L8/L16</f>
-        <v>2202.474701400835</v>
+        <f>L7/L16</f>
+        <v>9986.4185395484</v>
       </c>
       <c r="M18" s="35"/>
       <c r="N18" s="39" t="inlineStr">
@@ -6657,7 +6840,7 @@
       </c>
       <c r="L19" s="33">
         <f>L18-L13</f>
-        <v>989.334701400835</v>
+        <v>8773.2785395484</v>
       </c>
       <c r="M19" s="35"/>
       <c r="N19" s="39" t="inlineStr">
@@ -6669,12 +6852,12 @@
     <row r="20">
       <c r="K20" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC = BAC EVM − EAC</t>
+          <t xml:space="preserve">VAC = BAC total − EAC</t>
         </is>
       </c>
       <c r="L20" s="33">
-        <f>L8-L18</f>
-        <v>356.9452985991652</v>
+        <f>L7-L18</f>
+        <v>1234.7814604516</v>
       </c>
       <c r="M20" s="35"/>
       <c r="N20" s="39" t="str">
@@ -6692,7 +6875,7 @@
     <row r="24">
       <c r="K24" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• PV: 3 filas de devs (6 h/sem × 10 USD/h = 60 USD/sem c/u) durante 13 semanas + Azure B1 desde el deploy (29/08) + Claude Code/ChatGPT (3 × 20 USD/mes). La semana de reserva (05/11 → 12/11) es reserva de gestión y no entra.</t>
+          <t xml:space="preserve">• PV: 3 filas de devs (6 h/sem × 10 USD/h = 60 USD/sem c/u) + Azure B1 desde el deploy (29/08) + Claude Code/ChatGPT (3 × 20 USD/mes).</t>
         </is>
       </c>
     </row>
@@ -6706,7 +6889,7 @@
     <row r="26">
       <c r="K26" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EV = % completo × BAC EVM. % completo = horas estimadas de los paquetes de la WBS cerrados / 221,62 h de desarrollo. Semanal: 5,5 · 32,71 · 8,72 · 30,3 · 26,29 · 18,55 h (122,07 h).</t>
+          <t xml:space="preserve">• EV semanal: 8 · 30 · 20 · 21 · 21 · 23 h (total 123 h). Semana 1 floja, semana 2 se pone al día, semanas 3 a 6 un poco por encima del plan.</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6903,7 @@
     <row r="28">
       <c r="K28" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EAC, ETC y VAC usan el BAC de la línea base EVM (L8), la misma base que PV, EV y AC. BAC total del proyecto: 442 HH + infra e IA + 20 % de contingencia = 8.063,30 USD, sin CAPEX.</t>
+          <t xml:space="preserve">• EAC, ETC y VAC usan el BAC total del proyecto (11.221,20 USD: OPEX 12 sem + CAPEX + 20% de reservas), según el equipo.</t>
         </is>
       </c>
     </row>
@@ -6788,7 +6971,7 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equipo 11 · Semanas de jueves a jueves (06/08 → 05/11) · S1 = sem 1–6, S2 = 7–10, S3 = 11–13 · Reserva 05/11 → 12/11 fuera del BAC · Celdas amarillas = datos a editar</t>
+          <t xml:space="preserve">Equipo 11 · Semanas de jueves a jueves · Tarifa dev en Curva S!L6 · Celdas amarillas = datos a editar</t>
         </is>
       </c>
     </row>
@@ -6825,7 +7008,7 @@
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">% completo de la semana</t>
+          <t xml:space="preserve">EV mano de obra (USD)</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
@@ -6840,7 +7023,7 @@
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">EV total (USD) = % × BAC EVM</t>
+          <t xml:space="preserve">EV total (USD)</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
@@ -6865,7 +7048,7 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1 · Capacitación</t>
+          <t xml:space="preserve">Capacitación</t>
         </is>
       </c>
       <c r="D6" s="29">
@@ -6876,11 +7059,11 @@
         <v>18</v>
       </c>
       <c r="F6" s="47">
-        <v>5.5</v>
-      </c>
-      <c r="G6" s="53">
-        <f>F6/'Curva S'!$L$9</f>
-        <v>0.024817254760400684</v>
+        <v>8</v>
+      </c>
+      <c r="G6" s="45">
+        <f>F6*'Curva S'!$L$6</f>
+        <v>80</v>
       </c>
       <c r="H6" s="28">
         <f>PRESUPUESTO!B12+PRESUPUESTO!B13+PRESUPUESTO!B14</f>
@@ -6891,8 +7074,8 @@
         <v>60</v>
       </c>
       <c r="J6" s="45">
-        <f>G6*'Curva S'!$L$8</f>
-        <v>63.51777817886472</v>
+        <f>G6+H6</f>
+        <v>140</v>
       </c>
       <c r="K6" s="45">
         <f>E6*'Curva S'!$L$6+I6</f>
@@ -6900,7 +7083,7 @@
       </c>
       <c r="L6" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cierran 3.1.1, 3.1.3</t>
+          <t xml:space="preserve">Arranque flojo: se achicó el alcance de la capacitación y no se cerró ningún ticket antes del 15/08.</t>
         </is>
       </c>
     </row>
@@ -6915,7 +7098,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 1</t>
         </is>
       </c>
       <c r="D7" s="29">
@@ -6926,11 +7109,11 @@
         <v>18</v>
       </c>
       <c r="F7" s="47">
-        <v>32.71</v>
-      </c>
-      <c r="G7" s="53">
-        <f>F7/'Curva S'!$L$9</f>
-        <v>0.14759498240231025</v>
+        <v>30</v>
+      </c>
+      <c r="G7" s="45">
+        <f>F7*'Curva S'!$L$6</f>
+        <v>300</v>
       </c>
       <c r="H7" s="28">
         <f>PRESUPUESTO!C12+PRESUPUESTO!C13+PRESUPUESTO!C14</f>
@@ -6941,8 +7124,8 @@
         <v>0</v>
       </c>
       <c r="J7" s="45">
-        <f>G7*'Curva S'!$L$8</f>
-        <v>377.75754986012095</v>
+        <f>G7+H7</f>
+        <v>300</v>
       </c>
       <c r="K7" s="45">
         <f>E7*'Curva S'!$L$6+I7</f>
@@ -6950,7 +7133,7 @@
       </c>
       <c r="L7" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cierran 3.1.2, 3.2.1, 4.1.1, 4.1.3, 4.1.4, 4.2.1, 4.2.2, 4.2.3, 10.2.1</t>
+          <t xml:space="preserve">Se pone al día: capacitación cerrada el 16/08 (3 días tarde), setup de repos y autenticación Firebase.</t>
         </is>
       </c>
     </row>
@@ -6965,7 +7148,7 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 2</t>
         </is>
       </c>
       <c r="D8" s="29">
@@ -6976,11 +7159,11 @@
         <v>18</v>
       </c>
       <c r="F8" s="47">
-        <v>8.72</v>
-      </c>
-      <c r="G8" s="53">
-        <f>F8/'Curva S'!$L$9</f>
-        <v>0.039346629365580726</v>
+        <v>20</v>
+      </c>
+      <c r="G8" s="45">
+        <f>F8*'Curva S'!$L$6</f>
+        <v>200</v>
       </c>
       <c r="H8" s="28">
         <f>PRESUPUESTO!D12+PRESUPUESTO!D13+PRESUPUESTO!D14</f>
@@ -6991,8 +7174,8 @@
         <v>0</v>
       </c>
       <c r="J8" s="45">
-        <f>G8*'Curva S'!$L$8</f>
-        <v>100.70455013085463</v>
+        <f>G8+H8</f>
+        <v>200</v>
       </c>
       <c r="K8" s="45">
         <f>E8*'Curva S'!$L$6+I8</f>
@@ -7000,7 +7183,7 @@
       </c>
       <c r="L8" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cierran 3.2.2, 4.1.2, 6.1.1, 9.1.4</t>
+          <t xml:space="preserve">Modelo y API de partidos, CI y Docker; ritmo apenas por encima del plan.</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7198,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 3</t>
         </is>
       </c>
       <c r="D9" s="29">
@@ -7026,11 +7209,11 @@
         <v>18</v>
       </c>
       <c r="F9" s="47">
-        <v>30.3</v>
-      </c>
-      <c r="G9" s="53">
-        <f>F9/'Curva S'!$L$9</f>
-        <v>0.1367205125891165</v>
+        <v>21</v>
+      </c>
+      <c r="G9" s="45">
+        <f>F9*'Curva S'!$L$6</f>
+        <v>210</v>
       </c>
       <c r="H9" s="28">
         <f>PRESUPUESTO!E12+PRESUPUESTO!E13+PRESUPUESTO!E14</f>
@@ -7041,8 +7224,8 @@
         <v>13.14</v>
       </c>
       <c r="J9" s="45">
-        <f>G9*'Curva S'!$L$8</f>
-        <v>349.9252143308365</v>
+        <f>G9+H9</f>
+        <v>223.14</v>
       </c>
       <c r="K9" s="45">
         <f>E9*'Curva S'!$L$6+I9</f>
@@ -7050,7 +7233,7 @@
       </c>
       <c r="L9" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cierran 3.2.3, 4.2.5, 6.1.2, 6.1.5, 6.2.3, 6.3.5, 7.2.1, 9.1.1, 9.1.2, 9.1.3</t>
+          <t xml:space="preserve">Deploy de front (Vercel) y back (Azure) el 29/08, antes de lo previsto; swipe y detalle de partido.</t>
         </is>
       </c>
     </row>
@@ -7065,7 +7248,7 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1</t>
+          <t xml:space="preserve">Sprint 4</t>
         </is>
       </c>
       <c r="D10" s="29">
@@ -7076,11 +7259,11 @@
         <v>18</v>
       </c>
       <c r="F10" s="47">
-        <v>26.29</v>
-      </c>
-      <c r="G10" s="53">
-        <f>F10/'Curva S'!$L$9</f>
-        <v>0.11862647775471527</v>
+        <v>21</v>
+      </c>
+      <c r="G10" s="45">
+        <f>F10*'Curva S'!$L$6</f>
+        <v>210</v>
       </c>
       <c r="H10" s="28">
         <f>PRESUPUESTO!F12+PRESUPUESTO!F13+PRESUPUESTO!F14</f>
@@ -7091,8 +7274,8 @@
         <v>60</v>
       </c>
       <c r="J10" s="45">
-        <f>G10*'Curva S'!$L$8</f>
-        <v>303.6149796949734</v>
+        <f>G10+H10</f>
+        <v>270</v>
       </c>
       <c r="K10" s="45">
         <f>E10*'Curva S'!$L$6+I10</f>
@@ -7100,7 +7283,7 @@
       </c>
       <c r="L10" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cierran 5.1.2, 5.2.1, 6.1.3, 6.2.1, 6.2.4, 6.3.1, 6.3.2, 6.3.3, 7.2.2</t>
+          <t xml:space="preserve">Solicitudes, wizard de creación y "Tus partidos"; se adelanta trabajo de la etapa 2.</t>
         </is>
       </c>
     </row>
@@ -7115,7 +7298,7 @@
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve">S1 · CORTE (steering 1)</t>
+          <t xml:space="preserve">Sprint 5 · CORTE</t>
         </is>
       </c>
       <c r="D11" s="43">
@@ -7126,11 +7309,11 @@
         <v>18</v>
       </c>
       <c r="F11" s="47">
-        <v>18.55</v>
-      </c>
-      <c r="G11" s="53">
-        <f>F11/'Curva S'!$L$9</f>
-        <v>0.08370183196462413</v>
+        <v>23</v>
+      </c>
+      <c r="G11" s="46">
+        <f>F11*'Curva S'!$L$6</f>
+        <v>230</v>
       </c>
       <c r="H11" s="42">
         <f>PRESUPUESTO!G12+PRESUPUESTO!G13+PRESUPUESTO!G14</f>
@@ -7141,8 +7324,8 @@
         <v>0</v>
       </c>
       <c r="J11" s="46">
-        <f>G11*'Curva S'!$L$8</f>
-        <v>214.22814276689832</v>
+        <f>G11+H11</f>
+        <v>230</v>
       </c>
       <c r="K11" s="46">
         <f>E11*'Curva S'!$L$6+I11</f>
@@ -7150,7 +7333,7 @@
       </c>
       <c r="L11" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cierran 4.2.4, 5.1.3, 5.1.5, 5.2.4, 5.2.5, 6.2.2, 6.3.4, 6.4.1</t>
+          <t xml:space="preserve">Rating, perfil ajeno y landing; cierre con 1 ticket In Review + 4 Todo para el steering.</t>
         </is>
       </c>
     </row>
@@ -7165,7 +7348,7 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D12" s="29">
@@ -7199,7 +7382,7 @@
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D13" s="29">
@@ -7233,7 +7416,7 @@
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D14" s="29">
@@ -7267,7 +7450,7 @@
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S2 · MVP</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D15" s="29">
@@ -7301,7 +7484,7 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S3</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D16" s="29">
@@ -7335,7 +7518,7 @@
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">S3</t>
+          <t xml:space="preserve">Línea base</t>
         </is>
       </c>
       <c r="D17" s="29">
@@ -7359,80 +7542,46 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27">
-        <v>13</v>
-      </c>
-      <c r="B18" s="27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">05/11</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S3 · Fin del desarrollo</t>
-        </is>
-      </c>
-      <c r="D18" s="29">
-        <f>(PRESUPUESTO!N9+PRESUPUESTO!N10+PRESUPUESTO!N11)/'Curva S'!$L$6</f>
-        <v>18</v>
-      </c>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="28">
-        <f>PRESUPUESTO!N12+PRESUPUESTO!N13+PRESUPUESTO!N14</f>
-        <v>0</v>
-      </c>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27"/>
-      <c r="L18" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pendiente (línea base)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">Total al corte</t>
         </is>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="48">
+      <c r="B18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="48">
         <f>SUM(D6:D11)</f>
         <v>108</v>
       </c>
-      <c r="E19" s="48">
+      <c r="E18" s="48">
         <f>SUM(E6:E11)</f>
         <v>108</v>
       </c>
-      <c r="F19" s="48">
+      <c r="F18" s="48">
         <f>SUM(F6:F11)</f>
-        <v>122.07000000000001</v>
-      </c>
-      <c r="G19" s="53">
+        <v>123</v>
+      </c>
+      <c r="G18" s="49">
         <f>SUM(G6:G11)</f>
-        <v>0.5508076888367475</v>
-      </c>
-      <c r="H19" s="49">
+        <v>1230</v>
+      </c>
+      <c r="H18" s="49">
         <f>SUM(H6:H11)</f>
         <v>133.14</v>
       </c>
-      <c r="I19" s="49">
+      <c r="I18" s="49">
         <f>SUM(I6:I11)</f>
         <v>133.14</v>
       </c>
-      <c r="J19" s="49">
+      <c r="J18" s="49">
         <f>SUM(J6:J11)</f>
-        <v>1409.7482149625487</v>
-      </c>
-      <c r="K19" s="49">
+        <v>1363.14</v>
+      </c>
+      <c r="K18" s="49">
         <f>SUM(K6:K11)</f>
-        <v>1213.1399999999999</v>
-      </c>
-      <c r="L19" s="39" t="inlineStr">
+        <v>1213.14</v>
+      </c>
+      <c r="L18" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Semanas 1 a 6</t>
         </is>
@@ -7455,7 +7604,7 @@
     <row r="22">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Horas ganadas: horas estimadas (WBS v4) de los paquetes que cierran en la semana, según el Cronograma v4 §4. Total al corte: 122,07 h de 221,62 h de desarrollo. Los paquetes parciales no suman.</t>
+          <t xml:space="preserve">• Horas ganadas: horas de WBS entregadas en la semana. Total 123 h = 69 tickets Done + 1 In Review + 4 Todo de Linear.</t>
         </is>
       </c>
     </row>
@@ -7469,7 +7618,7 @@
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EV total = % completo de la semana × BAC EVM (Curva S!L8). AC total = horas reales × tarifa + Infra/IA facturados. Ambas columnas alimentan las filas 41 y 43 de PRESUPUESTO.</t>
+          <t xml:space="preserve">• EV total = EV mano de obra + Infra/IA consumidos. AC total = horas reales × tarifa + Infra/IA facturados. Ambas columnas alimentan las filas 41 y 43 de PRESUPUESTO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cambios y correcciones de presupuesto.
</commit_message>
<xml_diff>
--- a/outputs/SportMatch - Equipo 11 - EVM y Curva S.xlsx
+++ b/outputs/SportMatch - Equipo 11 - EVM y Curva S.xlsx
@@ -502,7 +502,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
@@ -624,6 +624,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="20" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -1676,73 +1679,12 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Curva S'!$B$5:$B$16</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>13/08</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>20/08</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>27/08</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>03/09</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>10/09</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>17/09</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>24/09</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>01/10</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>08/10</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>15/10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>22/10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>29/10</c:v>
-                </c:pt>
-              </c:strCache>
+              <c:f>'Curva S'!$B$5:$B$17</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>PRESUPUESTO!$B$44:$G$44</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>240</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>420</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>793.14</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1033.14</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1213.14</c:v>
-                </c:pt>
-              </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
@@ -1816,73 +1758,12 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Curva S'!$B$5:$B$16</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>13/08</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>20/08</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>27/08</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>03/09</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>10/09</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>17/09</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>24/09</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>01/10</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>08/10</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>15/10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>22/10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>29/10</c:v>
-                </c:pt>
-              </c:strCache>
+              <c:f>'Curva S'!$B$5:$B$17</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
               <c:f>PRESUPUESTO!$B$42:$G$42</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>140</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>440</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>640</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>863.14</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1133.14</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1363.14</c:v>
-                </c:pt>
-              </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
@@ -1907,91 +1788,12 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'Curva S'!$B$5:$B$16</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>13/08</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>20/08</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>27/08</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>03/09</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>10/09</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>17/09</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>24/09</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>01/10</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>08/10</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>15/10</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>22/10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>29/10</c:v>
-                </c:pt>
-              </c:strCache>
+              <c:f>'Curva S'!$B$5:$B$17</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>PRESUPUESTO!$B$40:$M$40</c:f>
-              <c:numCache>
-                <c:formatCode>#,##0</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>240</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>420</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>600</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>793.14</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1033.14</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1213.14</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1393.14</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1586.28</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1766.28</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>2006.28</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>2186.28</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>2379.42</c:v>
-                </c:pt>
-              </c:numCache>
+              <c:f>PRESUPUESTO!$B$40:$N$40</c:f>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
@@ -4079,7 +3881,9 @@
       <c r="M9" s="50">
         <v>60</v>
       </c>
-      <c r="N9" s="50"/>
+      <c r="N9" s="50">
+        <v>60</v>
+      </c>
       <c r="O9" s="50"/>
       <c r="P9" s="50"/>
       <c r="Q9" s="50"/>
@@ -4093,7 +3897,6 @@
       <c r="Y9" s="50"/>
       <c r="Z9" s="51">
         <f t="shared" ref="Z9:Z33" si="0">SUM(B9:Y9)</f>
-        <v>720</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
@@ -4138,7 +3941,9 @@
       <c r="M10" s="50">
         <v>60</v>
       </c>
-      <c r="N10" s="50"/>
+      <c r="N10" s="50">
+        <v>60</v>
+      </c>
       <c r="O10" s="50"/>
       <c r="P10" s="50"/>
       <c r="Q10" s="50"/>
@@ -4197,7 +4002,9 @@
       <c r="M11" s="50">
         <v>60</v>
       </c>
-      <c r="N11" s="50"/>
+      <c r="N11" s="50">
+        <v>60</v>
+      </c>
       <c r="O11" s="50"/>
       <c r="P11" s="50"/>
       <c r="Q11" s="50"/>
@@ -4907,7 +4714,6 @@
       </c>
       <c r="B34" s="52">
         <f t="shared" ref="B34:Z34" si="1">SUM(B9:B33)</f>
-        <v>240</v>
       </c>
       <c r="C34" s="52">
         <f t="shared" si="1"/>
@@ -5020,7 +4826,6 @@
       </c>
       <c r="D35" s="52">
         <f t="shared" ref="D35:G35" si="2">C35+D34</f>
-        <v>600</v>
       </c>
       <c r="E35" s="52">
         <f t="shared" si="2"/>
@@ -5036,47 +4841,37 @@
       </c>
       <c r="H35" s="52">
         <f t="shared" ref="H35" si="3">G35+H34</f>
-        <v>1393.14</v>
       </c>
       <c r="I35" s="52">
         <f t="shared" ref="I35" si="4">H35+I34</f>
-        <v>1586.28</v>
       </c>
       <c r="J35" s="52">
         <f t="shared" ref="J35" si="5">I35+J34</f>
-        <v>1766.28</v>
       </c>
       <c r="K35" s="52">
         <f t="shared" ref="K35" si="6">J35+K34</f>
-        <v>2006.28</v>
       </c>
       <c r="L35" s="52">
         <f t="shared" ref="L35" si="7">K35+L34</f>
-        <v>2186.28</v>
       </c>
       <c r="M35" s="52">
         <f t="shared" ref="M35" si="8">L35+M34</f>
-        <v>2379.42</v>
       </c>
       <c r="N35" s="52">
         <f t="shared" ref="N35" si="9">M35+N34</f>
-        <v>2379.42</v>
       </c>
       <c r="O35" s="52">
         <f t="shared" ref="O35" si="10">N35+O34</f>
-        <v>2379.42</v>
       </c>
       <c r="P35" s="52">
         <f t="shared" ref="P35" si="11">O35+P34</f>
-        <v>2379.42</v>
       </c>
       <c r="Q35" s="52">
         <f>P35+Q34</f>
-        <v>2379.42</v>
+        <v>2559.4199999999996</v>
       </c>
       <c r="R35" s="52">
         <f t="shared" ref="R35:W35" si="12">Q35+R34</f>
-        <v>2379.42</v>
       </c>
       <c r="S35" s="52">
         <f t="shared" si="12"/>
@@ -5100,11 +4895,11 @@
       </c>
       <c r="X35" s="52">
         <f>W35+X34</f>
-        <v>2379.42</v>
+        <v>2559.4199999999996</v>
       </c>
       <c r="Y35" s="52">
         <f>X35+Y34</f>
-        <v>2379.42</v>
+        <v>2559.4199999999996</v>
       </c>
     </row>
     <row r="38" spans="1:26" ht="16.5" x14ac:dyDescent="0.25">
@@ -5117,7 +4912,6 @@
       </c>
       <c r="C38" s="16">
         <f t="shared" ref="C38:G38" si="13">C34</f>
-        <v>180</v>
       </c>
       <c r="D38" s="16">
         <f t="shared" si="13"/>
@@ -5137,7 +4931,6 @@
       </c>
       <c r="H38" s="16">
         <f t="shared" ref="H38:Y38" si="14">H34</f>
-        <v>180</v>
       </c>
       <c r="I38" s="16">
         <f t="shared" si="14"/>
@@ -5149,7 +4942,6 @@
       </c>
       <c r="K38" s="16">
         <f t="shared" ref="K38:X38" si="15">K34</f>
-        <v>240</v>
       </c>
       <c r="L38" s="16">
         <f t="shared" si="15"/>
@@ -5177,7 +4969,6 @@
       </c>
       <c r="R38" s="16">
         <f t="shared" ref="R38:W38" si="16">R34</f>
-        <v>0</v>
       </c>
       <c r="S38" s="16">
         <f t="shared" si="16"/>
@@ -5221,7 +5012,6 @@
       </c>
       <c r="C39" s="22">
         <f t="shared" ref="C39:Y39" si="17">C38</f>
-        <v>180</v>
       </c>
       <c r="D39" s="22">
         <f t="shared" si="17"/>
@@ -5313,7 +5103,7 @@
       </c>
       <c r="Z39" s="20">
         <f>Z34</f>
-        <v>2379.42</v>
+        <v>2559.42</v>
       </c>
     </row>
     <row r="40" spans="1:26" x14ac:dyDescent="0.25">
@@ -5326,7 +5116,6 @@
       </c>
       <c r="C40" s="11">
         <f t="shared" ref="C40:G40" si="18">C35</f>
-        <v>420</v>
       </c>
       <c r="D40" s="11">
         <f>D35</f>
@@ -5346,7 +5135,6 @@
       </c>
       <c r="H40" s="11">
         <f t="shared" ref="H40:Y40" si="19">H35</f>
-        <v>1393.14</v>
       </c>
       <c r="I40" s="11">
         <f t="shared" si="19"/>
@@ -5358,7 +5146,6 @@
       </c>
       <c r="K40" s="11">
         <f t="shared" ref="K40:X40" si="20">K35</f>
-        <v>2006.28</v>
       </c>
       <c r="L40" s="11">
         <f t="shared" si="20"/>
@@ -5386,7 +5173,6 @@
       </c>
       <c r="R40" s="11">
         <f t="shared" ref="R40:W40" si="21">R35</f>
-        <v>2379.42</v>
       </c>
       <c r="S40" s="11">
         <f t="shared" si="21"/>
@@ -5423,27 +5209,27 @@
       </c>
       <c r="B41" s="21">
         <f>'Avance semanal'!J6</f>
-        <v>140</v>
+        <v>63.51777817886472</v>
       </c>
       <c r="C41" s="21">
         <f>'Avance semanal'!J7</f>
-        <v>300</v>
+        <v>377.75754986012095</v>
       </c>
       <c r="D41" s="21">
         <f>'Avance semanal'!J8</f>
-        <v>200</v>
+        <v>100.70455013085463</v>
       </c>
       <c r="E41" s="21">
         <f>'Avance semanal'!J9</f>
-        <v>223.14</v>
+        <v>349.9252143308365</v>
       </c>
       <c r="F41" s="21">
         <f>'Avance semanal'!J10</f>
-        <v>270</v>
+        <v>303.6149796949734</v>
       </c>
       <c r="G41" s="21">
         <f>'Avance semanal'!J11</f>
-        <v>230</v>
+        <v>233.05250248172547</v>
       </c>
       <c r="H41" s="21"/>
       <c r="I41" s="21"/>
@@ -5470,15 +5256,14 @@
       </c>
       <c r="B42" s="12">
         <f>IF(B41=0,NA(),B41)</f>
-        <v>140</v>
+        <v>63.51777817886472</v>
       </c>
       <c r="C42" s="12">
         <f>IF(C41=0,NA(),B42+C41)</f>
-        <v>440</v>
+        <v>441.27532803898566</v>
       </c>
       <c r="D42" s="12">
         <f t="shared" ref="D42:Y42" si="22">IF(D41=0,NA(),C42+D41)</f>
-        <v>640</v>
       </c>
       <c r="E42" s="12">
         <f t="shared" si="22"/>
@@ -5490,7 +5275,7 @@
       </c>
       <c r="G42" s="12">
         <f t="shared" si="22"/>
-        <v>1363.14</v>
+        <v>1428.5725746773758</v>
       </c>
       <c r="H42" s="12" t="e">
         <f t="shared" si="22"/>
@@ -5626,7 +5411,6 @@
       </c>
       <c r="D44" s="13">
         <f t="shared" ref="D44:Y44" si="23">IF(D41=0,NA(),C44+D43)</f>
-        <v>600</v>
       </c>
       <c r="E44" s="13">
         <f t="shared" si="23"/>
@@ -5719,7 +5503,6 @@
       </c>
       <c r="B45" s="14">
         <f t="shared" ref="B45:Y45" si="24">IFERROR(B42/B40,"-")</f>
-        <v>0.5833333333</v>
       </c>
       <c r="C45" s="14">
         <f t="shared" si="24"/>
@@ -5739,7 +5522,7 @@
       </c>
       <c r="G45" s="14">
         <f t="shared" si="24"/>
-        <v>1.1236460755</v>
+        <v>1.1775826159201541</v>
       </c>
       <c r="H45" s="14" t="str">
         <f t="shared" si="24"/>
@@ -5820,11 +5603,10 @@
       </c>
       <c r="B46" s="14">
         <f>IFERROR(B42/B44,"-")</f>
-        <v>0.5833333333</v>
+        <v>0.26465740907860297</v>
       </c>
       <c r="C46" s="14">
         <f t="shared" ref="C46:Y46" si="25">IFERROR(C42/C44,"-")</f>
-        <v>1.0476190476</v>
       </c>
       <c r="D46" s="14">
         <f t="shared" si="25"/>
@@ -5840,7 +5622,7 @@
       </c>
       <c r="G46" s="14">
         <f t="shared" si="25"/>
-        <v>1.1236460755</v>
+        <v>1.1775826159201541</v>
       </c>
       <c r="H46" s="14" t="str">
         <f t="shared" si="25"/>
@@ -5856,7 +5638,6 @@
       </c>
       <c r="K46" s="14" t="str">
         <f t="shared" ref="K46:X46" si="26">IFERROR(K42/K44,"-")</f>
-        <v>-</v>
       </c>
       <c r="L46" s="14" t="str">
         <f t="shared" si="26"/>
@@ -5884,7 +5665,6 @@
       </c>
       <c r="R46" s="14" t="str">
         <f t="shared" ref="R46:W46" si="27">IFERROR(R42/R44,"-")</f>
-        <v>-</v>
       </c>
       <c r="S46" s="14" t="str">
         <f t="shared" si="27"/>
@@ -6162,7 +5942,7 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equipo 11 · Corte 17/09/2026 (semana 6) · USD acumulados (devs + infra + IA) · Datos desde PRESUPUESTO y Avance semanal</t>
+          <t xml:space="preserve">Equipo 11 · Corte 17/09/2026 (semana 6, cierre del S1) · USD acumulados (devs + infra + IA) · Base: WBS y Cronograma v4 · Datos desde PRESUPUESTO y Avance semanal</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6010,7 @@
       </c>
       <c r="C5" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capacitación</t>
+          <t xml:space="preserve">S1 · Capacitación</t>
         </is>
       </c>
       <c r="D5" s="28">
@@ -6239,7 +6019,7 @@
       </c>
       <c r="E5" s="28">
         <f>IFERROR(PRESUPUESTO!B42,"")</f>
-        <v>140</v>
+        <v>63.51777817886472</v>
       </c>
       <c r="F5" s="28">
         <f>IFERROR(PRESUPUESTO!B44,"")</f>
@@ -6251,7 +6031,7 @@
       </c>
       <c r="H5" s="29">
         <f>SUM('Avance semanal'!$F$6:F6)</f>
-        <v>8</v>
+        <v>5.5</v>
       </c>
       <c r="I5" s="29">
         <f>SUM('Avance semanal'!$E$6:E6)</f>
@@ -6277,7 +6057,7 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 1</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D6" s="28">
@@ -6286,7 +6066,7 @@
       </c>
       <c r="E6" s="28">
         <f>IFERROR(PRESUPUESTO!C42,"")</f>
-        <v>440</v>
+        <v>441.27532803898566</v>
       </c>
       <c r="F6" s="28">
         <f>IFERROR(PRESUPUESTO!C44,"")</f>
@@ -6298,7 +6078,7 @@
       </c>
       <c r="H6" s="29">
         <f>SUM('Avance semanal'!$F$6:F7)</f>
-        <v>38</v>
+        <v>38.21</v>
       </c>
       <c r="I6" s="29">
         <f>SUM('Avance semanal'!$E$6:E7)</f>
@@ -6324,7 +6104,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 2</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D7" s="28">
@@ -6333,7 +6113,7 @@
       </c>
       <c r="E7" s="28">
         <f>IFERROR(PRESUPUESTO!D42,"")</f>
-        <v>640</v>
+        <v>541.9798781698403</v>
       </c>
       <c r="F7" s="28">
         <f>IFERROR(PRESUPUESTO!D44,"")</f>
@@ -6345,7 +6125,7 @@
       </c>
       <c r="H7" s="29">
         <f>SUM('Avance semanal'!$F$6:F8)</f>
-        <v>58</v>
+        <v>46.93</v>
       </c>
       <c r="I7" s="29">
         <f>SUM('Avance semanal'!$E$6:E8)</f>
@@ -6357,7 +6137,7 @@
         </is>
       </c>
       <c r="L7" s="31">
-        <v>11221.2</v>
+        <v>8063.3</v>
       </c>
     </row>
     <row r="8">
@@ -6371,7 +6151,7 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 3</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D8" s="28">
@@ -6380,7 +6160,7 @@
       </c>
       <c r="E8" s="28">
         <f>IFERROR(PRESUPUESTO!E42,"")</f>
-        <v>863.14</v>
+        <v>891.9050925006768</v>
       </c>
       <c r="F8" s="28">
         <f>IFERROR(PRESUPUESTO!E44,"")</f>
@@ -6392,7 +6172,7 @@
       </c>
       <c r="H8" s="29">
         <f>SUM('Avance semanal'!$F$6:F9)</f>
-        <v>79</v>
+        <v>77.23</v>
       </c>
       <c r="I8" s="29">
         <f>SUM('Avance semanal'!$E$6:E9)</f>
@@ -6405,7 +6185,7 @@
       </c>
       <c r="L8" s="38">
         <f>PRESUPUESTO!Z39</f>
-        <v>2379.42</v>
+        <v>2559.42</v>
       </c>
     </row>
     <row r="9">
@@ -6419,20 +6199,20 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 4</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D9" s="28">
         <f>PRESUPUESTO!F40</f>
-        <v>1033.14</v>
+        <v>1033.1399999999999</v>
       </c>
       <c r="E9" s="28">
         <f>IFERROR(PRESUPUESTO!F42,"")</f>
-        <v>1133.14</v>
+        <v>1195.5200721956503</v>
       </c>
       <c r="F9" s="28">
         <f>IFERROR(PRESUPUESTO!F44,"")</f>
-        <v>1033.14</v>
+        <v>1033.1399999999999</v>
       </c>
       <c r="G9" s="29">
         <f>SUM('Avance semanal'!$D$6:D10)</f>
@@ -6440,12 +6220,20 @@
       </c>
       <c r="H9" s="29">
         <f>SUM('Avance semanal'!$F$6:F10)</f>
-        <v>100</v>
+        <v>103.52000000000001</v>
       </c>
       <c r="I9" s="29">
         <f>SUM('Avance semanal'!$E$6:E10)</f>
         <v>90</v>
       </c>
+      <c r="K9" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Esfuerzo de desarrollo (h, Cronograma v4)</t>
+        </is>
+      </c>
+      <c r="L9" s="30">
+        <v>221.62</v>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="41">
@@ -6458,20 +6246,20 @@
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 5 · CORTE</t>
+          <t xml:space="preserve">S1 · CORTE (steering 1)</t>
         </is>
       </c>
       <c r="D10" s="42">
         <f>PRESUPUESTO!G40</f>
-        <v>1213.14</v>
+        <v>1213.1399999999999</v>
       </c>
       <c r="E10" s="42">
         <f>IFERROR(PRESUPUESTO!G42,"")</f>
-        <v>1363.14</v>
+        <v>1428.5725746773758</v>
       </c>
       <c r="F10" s="42">
         <f>IFERROR(PRESUPUESTO!G44,"")</f>
-        <v>1213.14</v>
+        <v>1213.1399999999999</v>
       </c>
       <c r="G10" s="43">
         <f>SUM('Avance semanal'!$D$6:D11)</f>
@@ -6479,7 +6267,7 @@
       </c>
       <c r="H10" s="43">
         <f>SUM('Avance semanal'!$F$6:F11)</f>
-        <v>123</v>
+        <v>123.70000000000002</v>
       </c>
       <c r="I10" s="43">
         <f>SUM('Avance semanal'!$E$6:E11)</f>
@@ -6517,12 +6305,12 @@
       </c>
       <c r="C11" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2</t>
         </is>
       </c>
       <c r="D11" s="28">
         <f>PRESUPUESTO!H40</f>
-        <v>1393.14</v>
+        <v>1393.1399999999999</v>
       </c>
       <c r="E11" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!H42,"")</f>
@@ -6545,10 +6333,10 @@
       </c>
       <c r="L11" s="38">
         <f>INDEX(PRESUPUESTO!$B$40:$Y$40,$L$5)</f>
-        <v>1213.14</v>
+        <v>1213.1399999999999</v>
       </c>
       <c r="M11" s="35">
-        <f>INDEX($G$5:$G$16,$L$5)</f>
+        <f>INDEX($G$5:$G$17,$L$5)</f>
         <v>108</v>
       </c>
       <c r="N11" s="39"/>
@@ -6564,12 +6352,12 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2</t>
         </is>
       </c>
       <c r="D12" s="28">
         <f>PRESUPUESTO!I40</f>
-        <v>1586.28</v>
+        <v>1586.2799999999997</v>
       </c>
       <c r="E12" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!I42,"")</f>
@@ -6592,11 +6380,11 @@
       </c>
       <c r="L12" s="38">
         <f>INDEX(PRESUPUESTO!$B$42:$Y$42,$L$5)</f>
-        <v>1363.14</v>
+        <v>1428.5725746773758</v>
       </c>
       <c r="M12" s="35">
-        <f>INDEX($H$5:$H$16,$L$5)</f>
-        <v>123</v>
+        <f>INDEX($H$5:$H$17,$L$5)</f>
+        <v>123.70000000000002</v>
       </c>
       <c r="N12" s="39"/>
     </row>
@@ -6611,12 +6399,12 @@
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2</t>
         </is>
       </c>
       <c r="D13" s="28">
         <f>PRESUPUESTO!J40</f>
-        <v>1766.28</v>
+        <v>1766.2799999999997</v>
       </c>
       <c r="E13" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!J42,"")</f>
@@ -6639,10 +6427,10 @@
       </c>
       <c r="L13" s="38">
         <f>INDEX(PRESUPUESTO!$B$44:$Y$44,$L$5)</f>
-        <v>1213.14</v>
+        <v>1213.1399999999999</v>
       </c>
       <c r="M13" s="35">
-        <f>INDEX($I$5:$I$16,$L$5)</f>
+        <f>INDEX($I$5:$I$17,$L$5)</f>
         <v>108</v>
       </c>
       <c r="N13" s="39"/>
@@ -6658,12 +6446,12 @@
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2 · MVP</t>
         </is>
       </c>
       <c r="D14" s="28">
         <f>PRESUPUESTO!K40</f>
-        <v>2006.28</v>
+        <v>2006.2799999999997</v>
       </c>
       <c r="E14" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!K42,"")</f>
@@ -6686,11 +6474,11 @@
       </c>
       <c r="L14" s="33">
         <f>L12-L13</f>
-        <v>150</v>
+        <v>215.43257467737567</v>
       </c>
       <c r="M14" s="35">
         <f>M12-M13</f>
-        <v>15</v>
+        <v>15.700000000000017</v>
       </c>
       <c r="N14" s="39" t="str">
         <f>IF(L14&gt;=0,"Bajo presupuesto","Sobre presupuesto")</f>
@@ -6708,12 +6496,12 @@
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S3</t>
         </is>
       </c>
       <c r="D15" s="28">
         <f>PRESUPUESTO!L40</f>
-        <v>2186.28</v>
+        <v>2186.2799999999997</v>
       </c>
       <c r="E15" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!L42,"")</f>
@@ -6736,11 +6524,11 @@
       </c>
       <c r="L15" s="33">
         <f>L12-L11</f>
-        <v>150</v>
+        <v>215.43257467737567</v>
       </c>
       <c r="M15" s="35">
         <f>M12-M11</f>
-        <v>15</v>
+        <v>15.700000000000017</v>
       </c>
       <c r="N15" s="39" t="str">
         <f>IF(L15&gt;=0,"Adelantado al plan","Atrasado")</f>
@@ -6758,12 +6546,12 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S3</t>
         </is>
       </c>
       <c r="D16" s="28">
         <f>PRESUPUESTO!M40</f>
-        <v>2379.42</v>
+        <v>2379.4199999999996</v>
       </c>
       <c r="E16" s="28" t="str">
         <f>IFERROR(PRESUPUESTO!M42,"")</f>
@@ -6786,7 +6574,7 @@
       </c>
       <c r="L16" s="34">
         <f>L12/L13</f>
-        <v>1.1236460755</v>
+        <v>1.1775826159201541</v>
       </c>
       <c r="M16" s="35"/>
       <c r="N16" s="39" t="str">
@@ -6795,6 +6583,35 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" s="27">
+        <v>13</v>
+      </c>
+      <c r="B17" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05/11</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 · Fin del desarrollo</t>
+        </is>
+      </c>
+      <c r="D17" s="28">
+        <f>PRESUPUESTO!N40</f>
+        <v>2559.4199999999996</v>
+      </c>
+      <c r="E17" s="28" t="str">
+        <f>IFERROR(PRESUPUESTO!N42,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="28" t="str">
+        <f>IFERROR(PRESUPUESTO!N44,"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="29">
+        <f>SUM('Avance semanal'!$D$6:D18)</f>
+        <v>234</v>
+      </c>
       <c r="K17" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">SPI = EV / PV</t>
@@ -6802,7 +6619,7 @@
       </c>
       <c r="L17" s="34">
         <f>L12/L11</f>
-        <v>1.1236460755</v>
+        <v>1.1775826159201541</v>
       </c>
       <c r="M17" s="35"/>
       <c r="N17" s="39" t="str">
@@ -6818,12 +6635,12 @@
       </c>
       <c r="K18" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">EAC = BAC total / CPI</t>
+          <t xml:space="preserve">EAC = BAC EVM / CPI</t>
         </is>
       </c>
       <c r="L18" s="33">
-        <f>L7/L16</f>
-        <v>9986.4185395484</v>
+        <f>L8/L16</f>
+        <v>2173.4526014551334</v>
       </c>
       <c r="M18" s="35"/>
       <c r="N18" s="39" t="inlineStr">
@@ -6840,7 +6657,7 @@
       </c>
       <c r="L19" s="33">
         <f>L18-L13</f>
-        <v>8773.2785395484</v>
+        <v>960.3126014551333</v>
       </c>
       <c r="M19" s="35"/>
       <c r="N19" s="39" t="inlineStr">
@@ -6852,12 +6669,12 @@
     <row r="20">
       <c r="K20" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">VAC = BAC total − EAC</t>
+          <t xml:space="preserve">VAC = BAC EVM − EAC</t>
         </is>
       </c>
       <c r="L20" s="33">
-        <f>L7-L18</f>
-        <v>1234.7814604516</v>
+        <f>L8-L18</f>
+        <v>385.9673985448667</v>
       </c>
       <c r="M20" s="35"/>
       <c r="N20" s="39" t="str">
@@ -6875,7 +6692,7 @@
     <row r="24">
       <c r="K24" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• PV: 3 filas de devs (6 h/sem × 10 USD/h = 60 USD/sem c/u) + Azure B1 desde el deploy (29/08) + Claude Code/ChatGPT (3 × 20 USD/mes).</t>
+          <t xml:space="preserve">• PV: 3 filas de devs (6 h/sem × 10 USD/h = 60 USD/sem c/u) durante 13 semanas + Azure B1 desde el deploy (29/08) + Claude Code/ChatGPT (3 × 20 USD/mes). La semana de reserva (05/11 → 12/11) es reserva de gestión y no entra.</t>
         </is>
       </c>
     </row>
@@ -6889,7 +6706,7 @@
     <row r="26">
       <c r="K26" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EV semanal: 8 · 30 · 20 · 21 · 21 · 23 h (total 123 h). Semana 1 floja, semana 2 se pone al día, semanas 3 a 6 un poco por encima del plan.</t>
+          <t xml:space="preserve">• EV = % completo × BAC EVM. % completo = horas estimadas de los paquetes de la WBS cerrados / 221,62 h de desarrollo. Semanal: 5,5 · 32,71 · 8,72 · 30,3 · 26,29 · 20,18 h (123,70 h).</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6720,7 @@
     <row r="28">
       <c r="K28" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EAC, ETC y VAC usan el BAC total del proyecto (11.221,20 USD: OPEX 12 sem + CAPEX + 20% de reservas), según el equipo.</t>
+          <t xml:space="preserve">• EAC, ETC y VAC usan el BAC de la línea base EVM (L8), la misma base que PV, EV y AC. BAC total del proyecto: 442 HH + infra e IA + 20 % de contingencia = 8.063,30 USD, sin CAPEX.</t>
         </is>
       </c>
     </row>
@@ -6971,7 +6788,7 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Equipo 11 · Semanas de jueves a jueves · Tarifa dev en Curva S!L6 · Celdas amarillas = datos a editar</t>
+          <t xml:space="preserve">Equipo 11 · Semanas de jueves a jueves (06/08 → 05/11) · S1 = sem 1–6, S2 = 7–10, S3 = 11–13 · Reserva 05/11 → 12/11 fuera del BAC · Celdas amarillas = datos a editar</t>
         </is>
       </c>
     </row>
@@ -7008,7 +6825,7 @@
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">EV mano de obra (USD)</t>
+          <t xml:space="preserve">% completo de la semana</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
@@ -7023,7 +6840,7 @@
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">EV total (USD)</t>
+          <t xml:space="preserve">EV total (USD) = % × BAC EVM</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
@@ -7048,7 +6865,7 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capacitación</t>
+          <t xml:space="preserve">S1 · Capacitación</t>
         </is>
       </c>
       <c r="D6" s="29">
@@ -7059,11 +6876,11 @@
         <v>18</v>
       </c>
       <c r="F6" s="47">
-        <v>8</v>
-      </c>
-      <c r="G6" s="45">
-        <f>F6*'Curva S'!$L$6</f>
-        <v>80</v>
+        <v>5.5</v>
+      </c>
+      <c r="G6" s="53">
+        <f>F6/'Curva S'!$L$9</f>
+        <v>0.024817254760400684</v>
       </c>
       <c r="H6" s="28">
         <f>PRESUPUESTO!B12+PRESUPUESTO!B13+PRESUPUESTO!B14</f>
@@ -7074,8 +6891,8 @@
         <v>60</v>
       </c>
       <c r="J6" s="45">
-        <f>G6+H6</f>
-        <v>140</v>
+        <f>G6*'Curva S'!$L$8</f>
+        <v>63.51777817886472</v>
       </c>
       <c r="K6" s="45">
         <f>E6*'Curva S'!$L$6+I6</f>
@@ -7083,7 +6900,7 @@
       </c>
       <c r="L6" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arranque flojo: se achicó el alcance de la capacitación y no se cerró ningún ticket antes del 15/08.</t>
+          <t xml:space="preserve">Cierran 3.1.1, 3.1.3</t>
         </is>
       </c>
     </row>
@@ -7098,7 +6915,7 @@
       </c>
       <c r="C7" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 1</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D7" s="29">
@@ -7109,11 +6926,11 @@
         <v>18</v>
       </c>
       <c r="F7" s="47">
-        <v>30</v>
-      </c>
-      <c r="G7" s="45">
-        <f>F7*'Curva S'!$L$6</f>
-        <v>300</v>
+        <v>32.71</v>
+      </c>
+      <c r="G7" s="53">
+        <f>F7/'Curva S'!$L$9</f>
+        <v>0.14759498240231025</v>
       </c>
       <c r="H7" s="28">
         <f>PRESUPUESTO!C12+PRESUPUESTO!C13+PRESUPUESTO!C14</f>
@@ -7124,8 +6941,8 @@
         <v>0</v>
       </c>
       <c r="J7" s="45">
-        <f>G7+H7</f>
-        <v>300</v>
+        <f>G7*'Curva S'!$L$8</f>
+        <v>377.75754986012095</v>
       </c>
       <c r="K7" s="45">
         <f>E7*'Curva S'!$L$6+I7</f>
@@ -7133,7 +6950,7 @@
       </c>
       <c r="L7" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Se pone al día: capacitación cerrada el 16/08 (3 días tarde), setup de repos y autenticación Firebase.</t>
+          <t xml:space="preserve">Cierran 3.1.2, 3.2.1, 4.1.1, 4.1.3, 4.1.4, 4.2.1, 4.2.2, 4.2.3, 10.2.1</t>
         </is>
       </c>
     </row>
@@ -7148,7 +6965,7 @@
       </c>
       <c r="C8" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 2</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D8" s="29">
@@ -7159,11 +6976,11 @@
         <v>18</v>
       </c>
       <c r="F8" s="47">
-        <v>20</v>
-      </c>
-      <c r="G8" s="45">
-        <f>F8*'Curva S'!$L$6</f>
-        <v>200</v>
+        <v>8.72</v>
+      </c>
+      <c r="G8" s="53">
+        <f>F8/'Curva S'!$L$9</f>
+        <v>0.039346629365580726</v>
       </c>
       <c r="H8" s="28">
         <f>PRESUPUESTO!D12+PRESUPUESTO!D13+PRESUPUESTO!D14</f>
@@ -7174,8 +6991,8 @@
         <v>0</v>
       </c>
       <c r="J8" s="45">
-        <f>G8+H8</f>
-        <v>200</v>
+        <f>G8*'Curva S'!$L$8</f>
+        <v>100.70455013085463</v>
       </c>
       <c r="K8" s="45">
         <f>E8*'Curva S'!$L$6+I8</f>
@@ -7183,7 +7000,7 @@
       </c>
       <c r="L8" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Modelo y API de partidos, CI y Docker; ritmo apenas por encima del plan.</t>
+          <t xml:space="preserve">Cierran 3.2.2, 4.1.2, 6.1.1, 9.1.4</t>
         </is>
       </c>
     </row>
@@ -7198,7 +7015,7 @@
       </c>
       <c r="C9" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 3</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D9" s="29">
@@ -7209,11 +7026,11 @@
         <v>18</v>
       </c>
       <c r="F9" s="47">
-        <v>21</v>
-      </c>
-      <c r="G9" s="45">
-        <f>F9*'Curva S'!$L$6</f>
-        <v>210</v>
+        <v>30.3</v>
+      </c>
+      <c r="G9" s="53">
+        <f>F9/'Curva S'!$L$9</f>
+        <v>0.1367205125891165</v>
       </c>
       <c r="H9" s="28">
         <f>PRESUPUESTO!E12+PRESUPUESTO!E13+PRESUPUESTO!E14</f>
@@ -7224,8 +7041,8 @@
         <v>13.14</v>
       </c>
       <c r="J9" s="45">
-        <f>G9+H9</f>
-        <v>223.14</v>
+        <f>G9*'Curva S'!$L$8</f>
+        <v>349.9252143308365</v>
       </c>
       <c r="K9" s="45">
         <f>E9*'Curva S'!$L$6+I9</f>
@@ -7233,7 +7050,7 @@
       </c>
       <c r="L9" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deploy de front (Vercel) y back (Azure) el 29/08, antes de lo previsto; swipe y detalle de partido.</t>
+          <t xml:space="preserve">Cierran 3.2.3, 4.2.5, 6.1.2, 6.1.5, 6.2.3, 6.3.5, 7.2.1, 9.1.1, 9.1.2, 9.1.3</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7065,7 @@
       </c>
       <c r="C10" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 4</t>
+          <t xml:space="preserve">S1</t>
         </is>
       </c>
       <c r="D10" s="29">
@@ -7259,11 +7076,11 @@
         <v>18</v>
       </c>
       <c r="F10" s="47">
-        <v>21</v>
-      </c>
-      <c r="G10" s="45">
-        <f>F10*'Curva S'!$L$6</f>
-        <v>210</v>
+        <v>26.29</v>
+      </c>
+      <c r="G10" s="53">
+        <f>F10/'Curva S'!$L$9</f>
+        <v>0.11862647775471527</v>
       </c>
       <c r="H10" s="28">
         <f>PRESUPUESTO!F12+PRESUPUESTO!F13+PRESUPUESTO!F14</f>
@@ -7274,8 +7091,8 @@
         <v>60</v>
       </c>
       <c r="J10" s="45">
-        <f>G10+H10</f>
-        <v>270</v>
+        <f>G10*'Curva S'!$L$8</f>
+        <v>303.6149796949734</v>
       </c>
       <c r="K10" s="45">
         <f>E10*'Curva S'!$L$6+I10</f>
@@ -7283,7 +7100,7 @@
       </c>
       <c r="L10" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solicitudes, wizard de creación y "Tus partidos"; se adelanta trabajo de la etapa 2.</t>
+          <t xml:space="preserve">Cierran 5.1.2, 5.2.1, 6.1.3, 6.2.1, 6.2.4, 6.3.1, 6.3.2, 6.3.3, 7.2.2</t>
         </is>
       </c>
     </row>
@@ -7298,7 +7115,7 @@
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sprint 5 · CORTE</t>
+          <t xml:space="preserve">S1 · CORTE (steering 1)</t>
         </is>
       </c>
       <c r="D11" s="43">
@@ -7309,11 +7126,11 @@
         <v>18</v>
       </c>
       <c r="F11" s="47">
-        <v>23</v>
-      </c>
-      <c r="G11" s="46">
-        <f>F11*'Curva S'!$L$6</f>
-        <v>230</v>
+        <v>20.18</v>
+      </c>
+      <c r="G11" s="53">
+        <f>F11/'Curva S'!$L$9</f>
+        <v>0.09105676382997924</v>
       </c>
       <c r="H11" s="42">
         <f>PRESUPUESTO!G12+PRESUPUESTO!G13+PRESUPUESTO!G14</f>
@@ -7324,8 +7141,8 @@
         <v>0</v>
       </c>
       <c r="J11" s="46">
-        <f>G11+H11</f>
-        <v>230</v>
+        <f>G11*'Curva S'!$L$8</f>
+        <v>233.05250248172547</v>
       </c>
       <c r="K11" s="46">
         <f>E11*'Curva S'!$L$6+I11</f>
@@ -7333,7 +7150,7 @@
       </c>
       <c r="L11" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rating, perfil ajeno y landing; cierre con 1 ticket In Review + 4 Todo para el steering.</t>
+          <t xml:space="preserve">Cierran 4.2.4, 5.1.3, 5.1.5, 5.2.4, 5.2.5, 6.2.2, 6.3.4, 6.4.1, 6.4.2</t>
         </is>
       </c>
     </row>
@@ -7348,7 +7165,7 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2</t>
         </is>
       </c>
       <c r="D12" s="29">
@@ -7382,7 +7199,7 @@
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2</t>
         </is>
       </c>
       <c r="D13" s="29">
@@ -7416,7 +7233,7 @@
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2</t>
         </is>
       </c>
       <c r="D14" s="29">
@@ -7450,7 +7267,7 @@
       </c>
       <c r="C15" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S2 · MVP</t>
         </is>
       </c>
       <c r="D15" s="29">
@@ -7484,7 +7301,7 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S3</t>
         </is>
       </c>
       <c r="D16" s="29">
@@ -7518,7 +7335,7 @@
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Línea base</t>
+          <t xml:space="preserve">S3</t>
         </is>
       </c>
       <c r="D17" s="29">
@@ -7542,46 +7359,80 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="27">
+        <v>13</v>
+      </c>
+      <c r="B18" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05/11</t>
+        </is>
+      </c>
+      <c r="C18" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 · Fin del desarrollo</t>
+        </is>
+      </c>
+      <c r="D18" s="29">
+        <f>(PRESUPUESTO!N9+PRESUPUESTO!N10+PRESUPUESTO!N11)/'Curva S'!$L$6</f>
+        <v>18</v>
+      </c>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="28">
+        <f>PRESUPUESTO!N12+PRESUPUESTO!N13+PRESUPUESTO!N14</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pendiente (línea base)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">Total al corte</t>
         </is>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="48">
+      <c r="B19" s="32"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="48">
         <f>SUM(D6:D11)</f>
         <v>108</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E19" s="48">
         <f>SUM(E6:E11)</f>
         <v>108</v>
       </c>
-      <c r="F18" s="48">
+      <c r="F19" s="48">
         <f>SUM(F6:F11)</f>
-        <v>123</v>
-      </c>
-      <c r="G18" s="49">
+        <v>123.70000000000002</v>
+      </c>
+      <c r="G19" s="53">
         <f>SUM(G6:G11)</f>
-        <v>1230</v>
-      </c>
-      <c r="H18" s="49">
+        <v>0.5581626207021027</v>
+      </c>
+      <c r="H19" s="49">
         <f>SUM(H6:H11)</f>
         <v>133.14</v>
       </c>
-      <c r="I18" s="49">
+      <c r="I19" s="49">
         <f>SUM(I6:I11)</f>
         <v>133.14</v>
       </c>
-      <c r="J18" s="49">
+      <c r="J19" s="49">
         <f>SUM(J6:J11)</f>
-        <v>1363.14</v>
-      </c>
-      <c r="K18" s="49">
+        <v>1428.5725746773758</v>
+      </c>
+      <c r="K19" s="49">
         <f>SUM(K6:K11)</f>
-        <v>1213.14</v>
-      </c>
-      <c r="L18" s="39" t="inlineStr">
+        <v>1213.1399999999999</v>
+      </c>
+      <c r="L19" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Semanas 1 a 6</t>
         </is>
@@ -7604,7 +7455,7 @@
     <row r="22">
       <c r="A22" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Horas ganadas: horas de WBS entregadas en la semana. Total 123 h = 69 tickets Done + 1 In Review + 4 Todo de Linear.</t>
+          <t xml:space="preserve">• Horas ganadas: horas estimadas (WBS v4) de los paquetes que cierran en la semana, según el Cronograma v4 §4. Total al corte: 123,70 h de 221,62 h de desarrollo. Los paquetes parciales no suman.</t>
         </is>
       </c>
     </row>
@@ -7618,7 +7469,7 @@
     <row r="24">
       <c r="A24" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">• EV total = EV mano de obra + Infra/IA consumidos. AC total = horas reales × tarifa + Infra/IA facturados. Ambas columnas alimentan las filas 41 y 43 de PRESUPUESTO.</t>
+          <t xml:space="preserve">• EV total = % completo de la semana × BAC EVM (Curva S!L8). AC total = horas reales × tarifa + Infra/IA facturados. Ambas columnas alimentan las filas 41 y 43 de PRESUPUESTO.</t>
         </is>
       </c>
     </row>

</xml_diff>